<commit_message>
📅 日报更新 2026-08-16 11:03
</commit_message>
<xml_diff>
--- a/data/exports/毛毛矩阵/dist_order_2026-08-16.xlsx
+++ b/data/exports/毛毛矩阵/dist_order_2026-08-16.xlsx
@@ -8904,7 +8904,7 @@
       </c>
       <c r="B148" s="0" t="inlineStr">
         <is>
-          <t>哈哈哈 </t>
+          <t>笃定，</t>
         </is>
       </c>
       <c r="C148" s="0" t="inlineStr">
@@ -10229,7 +10229,7 @@
       </c>
       <c r="B170" s="0" t="inlineStr">
         <is>
-          <t>天道酬勤</t>
+          <t>一叶知秋</t>
         </is>
       </c>
       <c r="C170" s="0" t="inlineStr">

</xml_diff>